<commit_message>
Daily slate 2026-05-12 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-10.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-10.xlsx
@@ -645,13 +645,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>5094</v>
+        <v>5100</v>
       </c>
       <c r="E8" t="n">
-        <v>816</v>
+        <v>818</v>
       </c>
       <c r="F8" t="n">
-        <v>4278</v>
+        <v>4282</v>
       </c>
       <c r="G8" t="n">
         <v>16</v>
@@ -1266,7 +1266,7 @@
         <v>0</v>
       </c>
       <c r="X3" t="n">
-        <v>21.9</v>
+        <v>22.1</v>
       </c>
       <c r="Y3" t="n">
         <v>662</v>
@@ -1342,7 +1342,7 @@
         <v>12.3</v>
       </c>
       <c r="Y4" t="n">
-        <v>1350</v>
+        <v>1356</v>
       </c>
       <c r="Z4" t="n">
         <v>62.5</v>
@@ -1633,7 +1633,7 @@
         <v>16</v>
       </c>
       <c r="Y7" t="n">
-        <v>5094</v>
+        <v>5100</v>
       </c>
       <c r="Z7" t="n">
         <v>64.59999999999999</v>

</xml_diff>